<commit_message>
Regenerate all workspaces: propagate filter toolbar + Name/Label toggle
Filter toolbar and Name/Label toggle were in the template but only socal-whp
was regenerated. Full regenerate propagates both to sdge-whp, sce-be, liwp,
nve-qar (output + docs). TODO: those three items moved to Done.
</commit_message>
<xml_diff>
--- a/output/nve-qar/workflow_master_inventory.xlsx
+++ b/output/nve-qar/workflow_master_inventory.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Forms" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Fields" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="FormRelationships" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ReferencedDataFields" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Workflows" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Triggers" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Actions" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="WorkflowFieldUsage" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="BusinessProcesses" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forms" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FormRelationships" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReferencedDataFields" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Triggers" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkflowFieldUsage" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BusinessProcesses" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Forms'!$A$3:$J$14</definedName>

</xml_diff>

<commit_message>
Regenerated LIWP and WHP
</commit_message>
<xml_diff>
--- a/output/nve-qar/workflow_master_inventory.xlsx
+++ b/output/nve-qar/workflow_master_inventory.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Forms" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Fields" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="FormRelationships" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ReferencedDataFields" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Workflows" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Triggers" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Actions" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="WorkflowFieldUsage" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="BusinessProcesses" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forms" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fields" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FormRelationships" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReferencedDataFields" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflows" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Triggers" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkflowFieldUsage" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BusinessProcesses" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Forms'!$A$3:$J$14</definedName>

</xml_diff>

<commit_message>
Parse WFEngine workflows from workspace exports, add workflow write-conflict detection
All five workspace baselines were re-exported by the platform's new workflow
engine, which carries workflows as a top-level Workflows[] array (Triggers/
Steps shape) instead of the old per-form embedded WorkflowConfigs. The parser
only read the old shape, so every workspace was silently reporting 0
workflows (111 dropped fleet-wide). parse_workspace_export now parses both
shapes through a shared _parse_wfengine() helper, normalizes WFEngine's
numeric enums to plain strings, and summarizes BuiltIn.SendEmail actions into
the same shape Legacy notifications use so narration covers both.

Also adds a field-write conflict check: the workflow-detail panel now warns
when a workflow writes a field that another workflow in the same workspace
also writes (a real race with no guaranteed run order), linking to the other
workflow. Scoped to write collisions only, not shared triggers.
</commit_message>
<xml_diff>
--- a/output/nve-qar/workflow_master_inventory.xlsx
+++ b/output/nve-qar/workflow_master_inventory.xlsx
@@ -26,7 +26,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Workflows'!$A$3:$M$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Triggers'!$A$3:$L$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Actions'!$A$3:$L$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'WorkflowFieldUsage'!$A$3:$G$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'BusinessProcesses'!$A$3:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -100,7 +99,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00ECEFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -29715,7 +29714,7 @@
     <row r="412" ht="22" customHeight="1">
       <c r="A412" s="10" t="inlineStr">
         <is>
-          <t>Measures::AdditionalFilter</t>
+          <t>Measures::AuditMeasure</t>
         </is>
       </c>
       <c r="B412" s="10" t="inlineStr">
@@ -29725,17 +29724,17 @@
       </c>
       <c r="C412" s="10" t="inlineStr">
         <is>
-          <t>AdditionalFilter</t>
+          <t>AuditMeasure</t>
         </is>
       </c>
       <c r="D412" s="10" t="inlineStr">
         <is>
-          <t>Additional Filter</t>
+          <t>Audit Measure</t>
         </is>
       </c>
       <c r="E412" s="10" t="inlineStr">
         <is>
-          <t>List</t>
+          <t>Boolean</t>
         </is>
       </c>
       <c r="F412" s="10" t="inlineStr"/>
@@ -29765,7 +29764,7 @@
     <row r="413" ht="22" customHeight="1">
       <c r="A413" s="10" t="inlineStr">
         <is>
-          <t>Measures::Deemed2BLkWSavings</t>
+          <t>Measures::CustomParameters</t>
         </is>
       </c>
       <c r="B413" s="10" t="inlineStr">
@@ -29775,17 +29774,17 @@
       </c>
       <c r="C413" s="10" t="inlineStr">
         <is>
-          <t>Deemed2BLkWSavings</t>
+          <t>CustomParameters</t>
         </is>
       </c>
       <c r="D413" s="10" t="inlineStr">
         <is>
-          <t>Deemed 2BL kW Savings</t>
+          <t>Custom Parameters</t>
         </is>
       </c>
       <c r="E413" s="10" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Boolean</t>
         </is>
       </c>
       <c r="F413" s="10" t="inlineStr"/>
@@ -29815,7 +29814,7 @@
     <row r="414" ht="22" customHeight="1">
       <c r="A414" s="10" t="inlineStr">
         <is>
-          <t>Measures::MeasureQuantityUnits</t>
+          <t>Measures::Cost</t>
         </is>
       </c>
       <c r="B414" s="10" t="inlineStr">
@@ -29825,17 +29824,17 @@
       </c>
       <c r="C414" s="10" t="inlineStr">
         <is>
-          <t>MeasureQuantityUnits</t>
+          <t>Cost</t>
         </is>
       </c>
       <c r="D414" s="10" t="inlineStr">
         <is>
-          <t>Quantity Units</t>
+          <t>Cost</t>
         </is>
       </c>
       <c r="E414" s="10" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Calculation</t>
         </is>
       </c>
       <c r="F414" s="10" t="inlineStr"/>
@@ -29865,7 +29864,7 @@
     <row r="415" ht="22" customHeight="1">
       <c r="A415" s="10" t="inlineStr">
         <is>
-          <t>Measures::MeasureVariant</t>
+          <t>Measures::MaterialCost</t>
         </is>
       </c>
       <c r="B415" s="10" t="inlineStr">
@@ -29875,17 +29874,17 @@
       </c>
       <c r="C415" s="10" t="inlineStr">
         <is>
-          <t>MeasureVariant</t>
+          <t>MaterialCost</t>
         </is>
       </c>
       <c r="D415" s="10" t="inlineStr">
         <is>
-          <t>Variant</t>
+          <t>Material Cost</t>
         </is>
       </c>
       <c r="E415" s="10" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="F415" s="10" t="inlineStr"/>
@@ -29915,7 +29914,7 @@
     <row r="416" ht="22" customHeight="1">
       <c r="A416" s="10" t="inlineStr">
         <is>
-          <t>Measures::MaterialCost</t>
+          <t>Measures::DeemedkWSavings</t>
         </is>
       </c>
       <c r="B416" s="10" t="inlineStr">
@@ -29925,12 +29924,12 @@
       </c>
       <c r="C416" s="10" t="inlineStr">
         <is>
-          <t>MaterialCost</t>
+          <t>DeemedkWSavings</t>
         </is>
       </c>
       <c r="D416" s="10" t="inlineStr">
         <is>
-          <t>Material Cost</t>
+          <t>Deemed kW Savings</t>
         </is>
       </c>
       <c r="E416" s="10" t="inlineStr">
@@ -29965,7 +29964,7 @@
     <row r="417" ht="22" customHeight="1">
       <c r="A417" s="10" t="inlineStr">
         <is>
-          <t>Measures::SnuggProName</t>
+          <t>Measures::ReserveAmount</t>
         </is>
       </c>
       <c r="B417" s="10" t="inlineStr">
@@ -29975,17 +29974,17 @@
       </c>
       <c r="C417" s="10" t="inlineStr">
         <is>
-          <t>SnuggProName</t>
+          <t>ReserveAmount</t>
         </is>
       </c>
       <c r="D417" s="10" t="inlineStr">
         <is>
-          <t>SnuggPro Name</t>
+          <t>Reserve Amount</t>
         </is>
       </c>
       <c r="E417" s="10" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="F417" s="10" t="inlineStr"/>
@@ -30015,7 +30014,7 @@
     <row r="418" ht="22" customHeight="1">
       <c r="A418" s="10" t="inlineStr">
         <is>
-          <t>Measures::Deemed2BLThermsSavings</t>
+          <t>Measures::LaborCost</t>
         </is>
       </c>
       <c r="B418" s="10" t="inlineStr">
@@ -30025,17 +30024,17 @@
       </c>
       <c r="C418" s="10" t="inlineStr">
         <is>
-          <t>Deemed2BLThermsSavings</t>
+          <t>LaborCost</t>
         </is>
       </c>
       <c r="D418" s="10" t="inlineStr">
         <is>
-          <t>Deemed 2BL Therms Savings</t>
+          <t>Labor Cost</t>
         </is>
       </c>
       <c r="E418" s="10" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="F418" s="10" t="inlineStr"/>
@@ -30065,7 +30064,7 @@
     <row r="419" ht="22" customHeight="1">
       <c r="A419" s="10" t="inlineStr">
         <is>
-          <t>Measures::MeasureGrouping</t>
+          <t>Measures::AdditionalFilter</t>
         </is>
       </c>
       <c r="B419" s="10" t="inlineStr">
@@ -30075,17 +30074,17 @@
       </c>
       <c r="C419" s="10" t="inlineStr">
         <is>
-          <t>MeasureGrouping</t>
+          <t>AdditionalFilter</t>
         </is>
       </c>
       <c r="D419" s="10" t="inlineStr">
         <is>
-          <t>Measure Grouping</t>
+          <t>Additional Filter</t>
         </is>
       </c>
       <c r="E419" s="10" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>List</t>
         </is>
       </c>
       <c r="F419" s="10" t="inlineStr"/>
@@ -30115,7 +30114,7 @@
     <row r="420" ht="22" customHeight="1">
       <c r="A420" s="10" t="inlineStr">
         <is>
-          <t>Measures::Deemed2BLGallonSavings</t>
+          <t>Measures::Deemed2BLkWSavings</t>
         </is>
       </c>
       <c r="B420" s="10" t="inlineStr">
@@ -30125,12 +30124,12 @@
       </c>
       <c r="C420" s="10" t="inlineStr">
         <is>
-          <t>Deemed2BLGallonSavings</t>
+          <t>Deemed2BLkWSavings</t>
         </is>
       </c>
       <c r="D420" s="10" t="inlineStr">
         <is>
-          <t>Deemed 2BL Gallon Savings</t>
+          <t>Deemed 2BL kW Savings</t>
         </is>
       </c>
       <c r="E420" s="10" t="inlineStr">
@@ -30165,7 +30164,7 @@
     <row r="421" ht="22" customHeight="1">
       <c r="A421" s="10" t="inlineStr">
         <is>
-          <t>Measures::MeasureReportGroupCode</t>
+          <t>Measures::MeasureQuantityUnits</t>
         </is>
       </c>
       <c r="B421" s="10" t="inlineStr">
@@ -30175,12 +30174,12 @@
       </c>
       <c r="C421" s="10" t="inlineStr">
         <is>
-          <t>MeasureReportGroupCode</t>
+          <t>MeasureQuantityUnits</t>
         </is>
       </c>
       <c r="D421" s="10" t="inlineStr">
         <is>
-          <t>Report Group Code</t>
+          <t>Quantity Units</t>
         </is>
       </c>
       <c r="E421" s="10" t="inlineStr">
@@ -30215,7 +30214,7 @@
     <row r="422" ht="22" customHeight="1">
       <c r="A422" s="10" t="inlineStr">
         <is>
-          <t>Measures::IOU</t>
+          <t>Measures::MeasureVariant</t>
         </is>
       </c>
       <c r="B422" s="10" t="inlineStr">
@@ -30225,12 +30224,12 @@
       </c>
       <c r="C422" s="10" t="inlineStr">
         <is>
-          <t>IOU</t>
+          <t>MeasureVariant</t>
         </is>
       </c>
       <c r="D422" s="10" t="inlineStr">
         <is>
-          <t>IOU</t>
+          <t>Variant</t>
         </is>
       </c>
       <c r="E422" s="10" t="inlineStr">
@@ -30265,7 +30264,7 @@
     <row r="423" ht="22" customHeight="1">
       <c r="A423" s="10" t="inlineStr">
         <is>
-          <t>Measures::DeemedkWSavings</t>
+          <t>Measures::SnuggProName</t>
         </is>
       </c>
       <c r="B423" s="10" t="inlineStr">
@@ -30275,17 +30274,17 @@
       </c>
       <c r="C423" s="10" t="inlineStr">
         <is>
-          <t>DeemedkWSavings</t>
+          <t>SnuggProName</t>
         </is>
       </c>
       <c r="D423" s="10" t="inlineStr">
         <is>
-          <t>Deemed kW Savings</t>
+          <t>SnuggPro Name</t>
         </is>
       </c>
       <c r="E423" s="10" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="F423" s="10" t="inlineStr"/>
@@ -30315,7 +30314,7 @@
     <row r="424" ht="22" customHeight="1">
       <c r="A424" s="10" t="inlineStr">
         <is>
-          <t>Measures::AuditMeasure</t>
+          <t>Measures::Deemed2BLThermsSavings</t>
         </is>
       </c>
       <c r="B424" s="10" t="inlineStr">
@@ -30325,17 +30324,17 @@
       </c>
       <c r="C424" s="10" t="inlineStr">
         <is>
-          <t>AuditMeasure</t>
+          <t>Deemed2BLThermsSavings</t>
         </is>
       </c>
       <c r="D424" s="10" t="inlineStr">
         <is>
-          <t>Audit Measure</t>
+          <t>Deemed 2BL Therms Savings</t>
         </is>
       </c>
       <c r="E424" s="10" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="F424" s="10" t="inlineStr"/>
@@ -30365,7 +30364,7 @@
     <row r="425" ht="22" customHeight="1">
       <c r="A425" s="10" t="inlineStr">
         <is>
-          <t>Measures::FuelType</t>
+          <t>Measures::MeasureGrouping</t>
         </is>
       </c>
       <c r="B425" s="10" t="inlineStr">
@@ -30375,12 +30374,12 @@
       </c>
       <c r="C425" s="10" t="inlineStr">
         <is>
-          <t>FuelType</t>
+          <t>MeasureGrouping</t>
         </is>
       </c>
       <c r="D425" s="10" t="inlineStr">
         <is>
-          <t>Fuel Type</t>
+          <t>Measure Grouping</t>
         </is>
       </c>
       <c r="E425" s="10" t="inlineStr">
@@ -30415,7 +30414,7 @@
     <row r="426" ht="22" customHeight="1">
       <c r="A426" s="10" t="inlineStr">
         <is>
-          <t>Measures::TotalCO2SavingsMT</t>
+          <t>Measures::Deemed2BLGallonSavings</t>
         </is>
       </c>
       <c r="B426" s="10" t="inlineStr">
@@ -30425,12 +30424,12 @@
       </c>
       <c r="C426" s="10" t="inlineStr">
         <is>
-          <t>TotalCO2SavingsMT</t>
+          <t>Deemed2BLGallonSavings</t>
         </is>
       </c>
       <c r="D426" s="10" t="inlineStr">
         <is>
-          <t>Total CO2 Savings (MT)</t>
+          <t>Deemed 2BL Gallon Savings</t>
         </is>
       </c>
       <c r="E426" s="10" t="inlineStr">
@@ -30465,7 +30464,7 @@
     <row r="427" ht="22" customHeight="1">
       <c r="A427" s="10" t="inlineStr">
         <is>
-          <t>Measures::DeemedThermsSavings</t>
+          <t>Measures::MeasureReportGroupCode</t>
         </is>
       </c>
       <c r="B427" s="10" t="inlineStr">
@@ -30475,12 +30474,12 @@
       </c>
       <c r="C427" s="10" t="inlineStr">
         <is>
-          <t>DeemedThermsSavings</t>
+          <t>MeasureReportGroupCode</t>
         </is>
       </c>
       <c r="D427" s="10" t="inlineStr">
         <is>
-          <t>Deemed Therms Savings</t>
+          <t>Report Group Code</t>
         </is>
       </c>
       <c r="E427" s="10" t="inlineStr">
@@ -30515,7 +30514,7 @@
     <row r="428" ht="22" customHeight="1">
       <c r="A428" s="10" t="inlineStr">
         <is>
-          <t>Measures::ExternalId</t>
+          <t>Measures::IOU</t>
         </is>
       </c>
       <c r="B428" s="10" t="inlineStr">
@@ -30525,12 +30524,12 @@
       </c>
       <c r="C428" s="10" t="inlineStr">
         <is>
-          <t>ExternalId</t>
+          <t>IOU</t>
         </is>
       </c>
       <c r="D428" s="10" t="inlineStr">
         <is>
-          <t>External ID</t>
+          <t>IOU</t>
         </is>
       </c>
       <c r="E428" s="10" t="inlineStr">
@@ -30565,7 +30564,7 @@
     <row r="429" ht="22" customHeight="1">
       <c r="A429" s="10" t="inlineStr">
         <is>
-          <t>Measures::DeemedkWhSavings</t>
+          <t>Measures::FuelType</t>
         </is>
       </c>
       <c r="B429" s="10" t="inlineStr">
@@ -30575,12 +30574,12 @@
       </c>
       <c r="C429" s="10" t="inlineStr">
         <is>
-          <t>DeemedkWhSavings</t>
+          <t>FuelType</t>
         </is>
       </c>
       <c r="D429" s="10" t="inlineStr">
         <is>
-          <t>Deemed kWh Savings</t>
+          <t>Fuel Type</t>
         </is>
       </c>
       <c r="E429" s="10" t="inlineStr">
@@ -30615,7 +30614,7 @@
     <row r="430" ht="22" customHeight="1">
       <c r="A430" s="10" t="inlineStr">
         <is>
-          <t>Measures::Capacity</t>
+          <t>Measures::TotalCO2SavingsMT</t>
         </is>
       </c>
       <c r="B430" s="10" t="inlineStr">
@@ -30625,12 +30624,12 @@
       </c>
       <c r="C430" s="10" t="inlineStr">
         <is>
-          <t>Capacity</t>
+          <t>TotalCO2SavingsMT</t>
         </is>
       </c>
       <c r="D430" s="10" t="inlineStr">
         <is>
-          <t>Capacity</t>
+          <t>Total CO2 Savings (MT)</t>
         </is>
       </c>
       <c r="E430" s="10" t="inlineStr">
@@ -30665,7 +30664,7 @@
     <row r="431" ht="22" customHeight="1">
       <c r="A431" s="10" t="inlineStr">
         <is>
-          <t>Measures::MeasureDownpayment</t>
+          <t>Measures::DeemedThermsSavings</t>
         </is>
       </c>
       <c r="B431" s="10" t="inlineStr">
@@ -30675,12 +30674,12 @@
       </c>
       <c r="C431" s="10" t="inlineStr">
         <is>
-          <t>MeasureDownpayment</t>
+          <t>DeemedThermsSavings</t>
         </is>
       </c>
       <c r="D431" s="10" t="inlineStr">
         <is>
-          <t>Down Payment</t>
+          <t>Deemed Therms Savings</t>
         </is>
       </c>
       <c r="E431" s="10" t="inlineStr">
@@ -30715,7 +30714,7 @@
     <row r="432" ht="22" customHeight="1">
       <c r="A432" s="10" t="inlineStr">
         <is>
-          <t>Measures::SavingsUnit</t>
+          <t>Measures::ExternalId</t>
         </is>
       </c>
       <c r="B432" s="10" t="inlineStr">
@@ -30725,12 +30724,12 @@
       </c>
       <c r="C432" s="10" t="inlineStr">
         <is>
-          <t>SavingsUnit</t>
+          <t>ExternalId</t>
         </is>
       </c>
       <c r="D432" s="10" t="inlineStr">
         <is>
-          <t>Savings Unit</t>
+          <t>External ID</t>
         </is>
       </c>
       <c r="E432" s="10" t="inlineStr">
@@ -30765,7 +30764,7 @@
     <row r="433" ht="22" customHeight="1">
       <c r="A433" s="10" t="inlineStr">
         <is>
-          <t>Measures::ReserveAmount</t>
+          <t>Measures::DeemedkWhSavings</t>
         </is>
       </c>
       <c r="B433" s="10" t="inlineStr">
@@ -30775,17 +30774,17 @@
       </c>
       <c r="C433" s="10" t="inlineStr">
         <is>
-          <t>ReserveAmount</t>
+          <t>DeemedkWhSavings</t>
         </is>
       </c>
       <c r="D433" s="10" t="inlineStr">
         <is>
-          <t>Reserve Amount</t>
+          <t>Deemed kWh Savings</t>
         </is>
       </c>
       <c r="E433" s="10" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="F433" s="10" t="inlineStr"/>
@@ -30815,7 +30814,7 @@
     <row r="434" ht="22" customHeight="1">
       <c r="A434" s="10" t="inlineStr">
         <is>
-          <t>Measures::BulkPurchase</t>
+          <t>Measures::Capacity</t>
         </is>
       </c>
       <c r="B434" s="10" t="inlineStr">
@@ -30825,12 +30824,12 @@
       </c>
       <c r="C434" s="10" t="inlineStr">
         <is>
-          <t>BulkPurchase</t>
+          <t>Capacity</t>
         </is>
       </c>
       <c r="D434" s="10" t="inlineStr">
         <is>
-          <t>Bulk Purchase</t>
+          <t>Capacity</t>
         </is>
       </c>
       <c r="E434" s="10" t="inlineStr">
@@ -30865,7 +30864,7 @@
     <row r="435" ht="22" customHeight="1">
       <c r="A435" s="10" t="inlineStr">
         <is>
-          <t>Measures::DeemedMMBTU</t>
+          <t>Measures::MeasureDownpayment</t>
         </is>
       </c>
       <c r="B435" s="10" t="inlineStr">
@@ -30875,12 +30874,12 @@
       </c>
       <c r="C435" s="10" t="inlineStr">
         <is>
-          <t>DeemedMMBTU</t>
+          <t>MeasureDownpayment</t>
         </is>
       </c>
       <c r="D435" s="10" t="inlineStr">
         <is>
-          <t>Deemed MMBTU</t>
+          <t>Down Payment</t>
         </is>
       </c>
       <c r="E435" s="10" t="inlineStr">
@@ -30915,7 +30914,7 @@
     <row r="436" ht="22" customHeight="1">
       <c r="A436" s="10" t="inlineStr">
         <is>
-          <t>Measures::LaborCost</t>
+          <t>Measures::SavingsUnit</t>
         </is>
       </c>
       <c r="B436" s="10" t="inlineStr">
@@ -30925,17 +30924,17 @@
       </c>
       <c r="C436" s="10" t="inlineStr">
         <is>
-          <t>LaborCost</t>
+          <t>SavingsUnit</t>
         </is>
       </c>
       <c r="D436" s="10" t="inlineStr">
         <is>
-          <t>Labor Cost</t>
+          <t>Savings Unit</t>
         </is>
       </c>
       <c r="E436" s="10" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="F436" s="10" t="inlineStr"/>
@@ -30965,7 +30964,7 @@
     <row r="437" ht="22" customHeight="1">
       <c r="A437" s="10" t="inlineStr">
         <is>
-          <t>Measures::ExistingFuelType</t>
+          <t>Measures::BulkPurchase</t>
         </is>
       </c>
       <c r="B437" s="10" t="inlineStr">
@@ -30975,12 +30974,12 @@
       </c>
       <c r="C437" s="10" t="inlineStr">
         <is>
-          <t>ExistingFuelType</t>
+          <t>BulkPurchase</t>
         </is>
       </c>
       <c r="D437" s="10" t="inlineStr">
         <is>
-          <t>Existing Fuel Type</t>
+          <t>Bulk Purchase</t>
         </is>
       </c>
       <c r="E437" s="10" t="inlineStr">
@@ -31015,7 +31014,7 @@
     <row r="438" ht="22" customHeight="1">
       <c r="A438" s="10" t="inlineStr">
         <is>
-          <t>Measures::Category</t>
+          <t>Measures::DeemedMMBTU</t>
         </is>
       </c>
       <c r="B438" s="10" t="inlineStr">
@@ -31025,12 +31024,12 @@
       </c>
       <c r="C438" s="10" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>DeemedMMBTU</t>
         </is>
       </c>
       <c r="D438" s="10" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Deemed MMBTU</t>
         </is>
       </c>
       <c r="E438" s="10" t="inlineStr">
@@ -31065,7 +31064,7 @@
     <row r="439" ht="22" customHeight="1">
       <c r="A439" s="10" t="inlineStr">
         <is>
-          <t>Measures::MeasureCostNTE</t>
+          <t>Measures::ExistingFuelType</t>
         </is>
       </c>
       <c r="B439" s="10" t="inlineStr">
@@ -31075,12 +31074,12 @@
       </c>
       <c r="C439" s="10" t="inlineStr">
         <is>
-          <t>MeasureCostNTE</t>
+          <t>ExistingFuelType</t>
         </is>
       </c>
       <c r="D439" s="10" t="inlineStr">
         <is>
-          <t>Measure Cost (Not To Exceed)</t>
+          <t>Existing Fuel Type</t>
         </is>
       </c>
       <c r="E439" s="10" t="inlineStr">
@@ -31115,7 +31114,7 @@
     <row r="440" ht="22" customHeight="1">
       <c r="A440" s="10" t="inlineStr">
         <is>
-          <t>Measures::EULYears</t>
+          <t>Measures::Category</t>
         </is>
       </c>
       <c r="B440" s="10" t="inlineStr">
@@ -31125,12 +31124,12 @@
       </c>
       <c r="C440" s="10" t="inlineStr">
         <is>
-          <t>EULYears</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="D440" s="10" t="inlineStr">
         <is>
-          <t>EUL (Years)</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="E440" s="10" t="inlineStr">
@@ -31165,7 +31164,7 @@
     <row r="441" ht="22" customHeight="1">
       <c r="A441" s="10" t="inlineStr">
         <is>
-          <t>Measures::AFUE</t>
+          <t>Measures::MeasureCostNTE</t>
         </is>
       </c>
       <c r="B441" s="10" t="inlineStr">
@@ -31175,12 +31174,12 @@
       </c>
       <c r="C441" s="10" t="inlineStr">
         <is>
-          <t>AFUE</t>
+          <t>MeasureCostNTE</t>
         </is>
       </c>
       <c r="D441" s="10" t="inlineStr">
         <is>
-          <t>AFUE</t>
+          <t>Measure Cost (Not To Exceed)</t>
         </is>
       </c>
       <c r="E441" s="10" t="inlineStr">
@@ -31215,7 +31214,7 @@
     <row r="442" ht="22" customHeight="1">
       <c r="A442" s="10" t="inlineStr">
         <is>
-          <t>Measures::UEF</t>
+          <t>Measures::EULYears</t>
         </is>
       </c>
       <c r="B442" s="10" t="inlineStr">
@@ -31225,12 +31224,12 @@
       </c>
       <c r="C442" s="10" t="inlineStr">
         <is>
-          <t>UEF</t>
+          <t>EULYears</t>
         </is>
       </c>
       <c r="D442" s="10" t="inlineStr">
         <is>
-          <t>UEF</t>
+          <t>EUL (Years)</t>
         </is>
       </c>
       <c r="E442" s="10" t="inlineStr">
@@ -31265,7 +31264,7 @@
     <row r="443" ht="22" customHeight="1">
       <c r="A443" s="10" t="inlineStr">
         <is>
-          <t>Measures::Variation</t>
+          <t>Measures::AFUE</t>
         </is>
       </c>
       <c r="B443" s="10" t="inlineStr">
@@ -31275,12 +31274,12 @@
       </c>
       <c r="C443" s="10" t="inlineStr">
         <is>
-          <t>Variation</t>
+          <t>AFUE</t>
         </is>
       </c>
       <c r="D443" s="10" t="inlineStr">
         <is>
-          <t>Variation</t>
+          <t>AFUE</t>
         </is>
       </c>
       <c r="E443" s="10" t="inlineStr">
@@ -31315,7 +31314,7 @@
     <row r="444" ht="22" customHeight="1">
       <c r="A444" s="10" t="inlineStr">
         <is>
-          <t>Measures::InsulationRValue</t>
+          <t>Measures::UEF</t>
         </is>
       </c>
       <c r="B444" s="10" t="inlineStr">
@@ -31325,12 +31324,12 @@
       </c>
       <c r="C444" s="10" t="inlineStr">
         <is>
-          <t>InsulationRValue</t>
+          <t>UEF</t>
         </is>
       </c>
       <c r="D444" s="10" t="inlineStr">
         <is>
-          <t>R-Value</t>
+          <t>UEF</t>
         </is>
       </c>
       <c r="E444" s="10" t="inlineStr">
@@ -31365,7 +31364,7 @@
     <row r="445" ht="22" customHeight="1">
       <c r="A445" s="10" t="inlineStr">
         <is>
-          <t>Measures::Deemed2BLkWhSavings</t>
+          <t>Measures::Variation</t>
         </is>
       </c>
       <c r="B445" s="10" t="inlineStr">
@@ -31375,12 +31374,12 @@
       </c>
       <c r="C445" s="10" t="inlineStr">
         <is>
-          <t>Deemed2BLkWhSavings</t>
+          <t>Variation</t>
         </is>
       </c>
       <c r="D445" s="10" t="inlineStr">
         <is>
-          <t>Deemed 2BL kWh Savings</t>
+          <t>Variation</t>
         </is>
       </c>
       <c r="E445" s="10" t="inlineStr">
@@ -31415,7 +31414,7 @@
     <row r="446" ht="22" customHeight="1">
       <c r="A446" s="10" t="inlineStr">
         <is>
-          <t>Measures::ReportMeasureName</t>
+          <t>Measures::InsulationRValue</t>
         </is>
       </c>
       <c r="B446" s="10" t="inlineStr">
@@ -31425,12 +31424,12 @@
       </c>
       <c r="C446" s="10" t="inlineStr">
         <is>
-          <t>ReportMeasureName</t>
+          <t>InsulationRValue</t>
         </is>
       </c>
       <c r="D446" s="10" t="inlineStr">
         <is>
-          <t>Report Measure Name</t>
+          <t>R-Value</t>
         </is>
       </c>
       <c r="E446" s="10" t="inlineStr">
@@ -31465,7 +31464,7 @@
     <row r="447" ht="22" customHeight="1">
       <c r="A447" s="10" t="inlineStr">
         <is>
-          <t>Measures::PathRestriction</t>
+          <t>Measures::Deemed2BLkWhSavings</t>
         </is>
       </c>
       <c r="B447" s="10" t="inlineStr">
@@ -31475,12 +31474,12 @@
       </c>
       <c r="C447" s="10" t="inlineStr">
         <is>
-          <t>PathRestriction</t>
+          <t>Deemed2BLkWhSavings</t>
         </is>
       </c>
       <c r="D447" s="10" t="inlineStr">
         <is>
-          <t>Path Restriction</t>
+          <t>Deemed 2BL kWh Savings</t>
         </is>
       </c>
       <c r="E447" s="10" t="inlineStr">
@@ -31515,7 +31514,7 @@
     <row r="448" ht="22" customHeight="1">
       <c r="A448" s="10" t="inlineStr">
         <is>
-          <t>Measures::EULMonths</t>
+          <t>Measures::ReportMeasureName</t>
         </is>
       </c>
       <c r="B448" s="10" t="inlineStr">
@@ -31525,12 +31524,12 @@
       </c>
       <c r="C448" s="10" t="inlineStr">
         <is>
-          <t>EULMonths</t>
+          <t>ReportMeasureName</t>
         </is>
       </c>
       <c r="D448" s="10" t="inlineStr">
         <is>
-          <t>EUL (Months)</t>
+          <t>Report Measure Name</t>
         </is>
       </c>
       <c r="E448" s="10" t="inlineStr">
@@ -31565,7 +31564,7 @@
     <row r="449" ht="22" customHeight="1">
       <c r="A449" s="10" t="inlineStr">
         <is>
-          <t>Measures::MeasureReportGroup</t>
+          <t>Measures::PathRestriction</t>
         </is>
       </c>
       <c r="B449" s="10" t="inlineStr">
@@ -31575,12 +31574,12 @@
       </c>
       <c r="C449" s="10" t="inlineStr">
         <is>
-          <t>MeasureReportGroup</t>
+          <t>PathRestriction</t>
         </is>
       </c>
       <c r="D449" s="10" t="inlineStr">
         <is>
-          <t>Measure Report Group</t>
+          <t>Path Restriction</t>
         </is>
       </c>
       <c r="E449" s="10" t="inlineStr">
@@ -31615,7 +31614,7 @@
     <row r="450" ht="22" customHeight="1">
       <c r="A450" s="10" t="inlineStr">
         <is>
-          <t>Measures::Tons</t>
+          <t>Measures::EULMonths</t>
         </is>
       </c>
       <c r="B450" s="10" t="inlineStr">
@@ -31625,12 +31624,12 @@
       </c>
       <c r="C450" s="10" t="inlineStr">
         <is>
-          <t>Tons</t>
+          <t>EULMonths</t>
         </is>
       </c>
       <c r="D450" s="10" t="inlineStr">
         <is>
-          <t>Tons</t>
+          <t>EUL (Months)</t>
         </is>
       </c>
       <c r="E450" s="10" t="inlineStr">
@@ -31665,7 +31664,7 @@
     <row r="451" ht="22" customHeight="1">
       <c r="A451" s="10" t="inlineStr">
         <is>
-          <t>Measures::HVACType</t>
+          <t>Measures::MeasureReportGroup</t>
         </is>
       </c>
       <c r="B451" s="10" t="inlineStr">
@@ -31675,12 +31674,12 @@
       </c>
       <c r="C451" s="10" t="inlineStr">
         <is>
-          <t>HVACType</t>
+          <t>MeasureReportGroup</t>
         </is>
       </c>
       <c r="D451" s="10" t="inlineStr">
         <is>
-          <t>HVAC Type</t>
+          <t>Measure Report Group</t>
         </is>
       </c>
       <c r="E451" s="10" t="inlineStr">
@@ -31715,7 +31714,7 @@
     <row r="452" ht="22" customHeight="1">
       <c r="A452" s="10" t="inlineStr">
         <is>
-          <t>Measures::Cost</t>
+          <t>Measures::Tons</t>
         </is>
       </c>
       <c r="B452" s="10" t="inlineStr">
@@ -31725,17 +31724,17 @@
       </c>
       <c r="C452" s="10" t="inlineStr">
         <is>
-          <t>Cost</t>
+          <t>Tons</t>
         </is>
       </c>
       <c r="D452" s="10" t="inlineStr">
         <is>
-          <t>Cost</t>
+          <t>Tons</t>
         </is>
       </c>
       <c r="E452" s="10" t="inlineStr">
         <is>
-          <t>Calculation</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="F452" s="10" t="inlineStr"/>
@@ -31765,7 +31764,7 @@
     <row r="453" ht="22" customHeight="1">
       <c r="A453" s="10" t="inlineStr">
         <is>
-          <t>Measures::ReportMeasureCategory</t>
+          <t>Measures::HVACType</t>
         </is>
       </c>
       <c r="B453" s="10" t="inlineStr">
@@ -31775,12 +31774,12 @@
       </c>
       <c r="C453" s="10" t="inlineStr">
         <is>
-          <t>ReportMeasureCategory</t>
+          <t>HVACType</t>
         </is>
       </c>
       <c r="D453" s="10" t="inlineStr">
         <is>
-          <t>Report Measure Category</t>
+          <t>HVAC Type</t>
         </is>
       </c>
       <c r="E453" s="10" t="inlineStr">
@@ -31815,7 +31814,7 @@
     <row r="454" ht="22" customHeight="1">
       <c r="A454" s="10" t="inlineStr">
         <is>
-          <t>Measures::CostUnit</t>
+          <t>Measures::ReportMeasureCategory</t>
         </is>
       </c>
       <c r="B454" s="10" t="inlineStr">
@@ -31825,12 +31824,12 @@
       </c>
       <c r="C454" s="10" t="inlineStr">
         <is>
-          <t>CostUnit</t>
+          <t>ReportMeasureCategory</t>
         </is>
       </c>
       <c r="D454" s="10" t="inlineStr">
         <is>
-          <t>Cost Unit</t>
+          <t>Report Measure Category</t>
         </is>
       </c>
       <c r="E454" s="10" t="inlineStr">
@@ -31865,7 +31864,7 @@
     <row r="455" ht="22" customHeight="1">
       <c r="A455" s="10" t="inlineStr">
         <is>
-          <t>Measures::MeasureFilter</t>
+          <t>Measures::CostUnit</t>
         </is>
       </c>
       <c r="B455" s="10" t="inlineStr">
@@ -31875,12 +31874,12 @@
       </c>
       <c r="C455" s="10" t="inlineStr">
         <is>
-          <t>MeasureFilter</t>
+          <t>CostUnit</t>
         </is>
       </c>
       <c r="D455" s="10" t="inlineStr">
         <is>
-          <t>Measure Filter</t>
+          <t>Cost Unit</t>
         </is>
       </c>
       <c r="E455" s="10" t="inlineStr">
@@ -31915,7 +31914,7 @@
     <row r="456" ht="22" customHeight="1">
       <c r="A456" s="10" t="inlineStr">
         <is>
-          <t>Measures::SnuggProCode</t>
+          <t>Measures::MeasureFilter</t>
         </is>
       </c>
       <c r="B456" s="10" t="inlineStr">
@@ -31925,12 +31924,12 @@
       </c>
       <c r="C456" s="10" t="inlineStr">
         <is>
-          <t>SnuggProCode</t>
+          <t>MeasureFilter</t>
         </is>
       </c>
       <c r="D456" s="10" t="inlineStr">
         <is>
-          <t>SnuggPro Code</t>
+          <t>Measure Filter</t>
         </is>
       </c>
       <c r="E456" s="10" t="inlineStr">
@@ -31965,7 +31964,7 @@
     <row r="457" ht="22" customHeight="1">
       <c r="A457" s="10" t="inlineStr">
         <is>
-          <t>Measures::MeasureTypeCode</t>
+          <t>Measures::SnuggProCode</t>
         </is>
       </c>
       <c r="B457" s="10" t="inlineStr">
@@ -31975,12 +31974,12 @@
       </c>
       <c r="C457" s="10" t="inlineStr">
         <is>
-          <t>MeasureTypeCode</t>
+          <t>SnuggProCode</t>
         </is>
       </c>
       <c r="D457" s="10" t="inlineStr">
         <is>
-          <t>Measure Type Code</t>
+          <t>SnuggPro Code</t>
         </is>
       </c>
       <c r="E457" s="10" t="inlineStr">
@@ -32015,7 +32014,7 @@
     <row r="458" ht="22" customHeight="1">
       <c r="A458" s="10" t="inlineStr">
         <is>
-          <t>Measures::DetailedHVACType</t>
+          <t>Measures::MeasureTypeCode</t>
         </is>
       </c>
       <c r="B458" s="10" t="inlineStr">
@@ -32025,12 +32024,12 @@
       </c>
       <c r="C458" s="10" t="inlineStr">
         <is>
-          <t>DetailedHVACType</t>
+          <t>MeasureTypeCode</t>
         </is>
       </c>
       <c r="D458" s="10" t="inlineStr">
         <is>
-          <t>Detailed HVAC Type</t>
+          <t>Measure Type Code</t>
         </is>
       </c>
       <c r="E458" s="10" t="inlineStr">
@@ -32065,7 +32064,7 @@
     <row r="459" ht="22" customHeight="1">
       <c r="A459" s="10" t="inlineStr">
         <is>
-          <t>Measures::CustomParameters</t>
+          <t>Measures::DetailedHVACType</t>
         </is>
       </c>
       <c r="B459" s="10" t="inlineStr">
@@ -32075,17 +32074,17 @@
       </c>
       <c r="C459" s="10" t="inlineStr">
         <is>
-          <t>CustomParameters</t>
+          <t>DetailedHVACType</t>
         </is>
       </c>
       <c r="D459" s="10" t="inlineStr">
         <is>
-          <t>Custom Parameters</t>
+          <t>Detailed HVAC Type</t>
         </is>
       </c>
       <c r="E459" s="10" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="F459" s="10" t="inlineStr"/>
@@ -40697,7 +40696,7 @@
           <t>Dispatch to User</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr"/>
+      <c r="C5" s="10" t="n"/>
       <c r="D5" s="10" t="inlineStr">
         <is>
           <t>Runs when a new 895 - Installation / Warranty record is created.</t>
@@ -40705,7 +40704,7 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Legacy</t>
+          <t>WFEngine</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr"/>
@@ -40721,7 +40720,11 @@
         </is>
       </c>
       <c r="J5" s="10" t="inlineStr"/>
-      <c r="K5" s="10" t="inlineStr"/>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>6ab03969-872f-6878-a60c-3a226ee16f94</t>
+        </is>
+      </c>
       <c r="L5" s="10" t="inlineStr">
         <is>
           <t>qualified_appliance_replacement.json</t>
@@ -40920,8 +40923,14 @@
           <t>Create</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr"/>
-      <c r="H5" s="10" t="inlineStr"/>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Post-processing</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="I5" s="10" t="inlineStr"/>
       <c r="J5" s="10" t="inlineStr"/>
       <c r="K5" s="10" t="inlineStr"/>
@@ -41093,20 +41102,24 @@
           <t>895_DISPATCH_TO_USER</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr"/>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Send Email</t>
+        </is>
+      </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>QAR Installation {ProjectNumber} - {AddressStreet1}</t>
+          <t>Send Email</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Notification</t>
+          <t>BuiltIn.SendEmail</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Communication</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr"/>
@@ -41115,7 +41128,7 @@
       <c r="I5" s="10" t="inlineStr"/>
       <c r="J5" s="10" t="inlineStr">
         <is>
-          <t>To: {AssignedUserEmail} · Subject: QAR Installation {ProjectNumber} - {AddressStreet1}</t>
+          <t>To: AssignedUserEmail · Subject: QAR Installation {{ProjectNumber}} - {{AddressStreet1}}</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
@@ -41137,7 +41150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -41230,356 +41243,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>895_DISPATCH_TO_USER</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>895 - Installation / Warranty</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>AddressCity</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>Notification template</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr"/>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>895_DISPATCH_TO_USER</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>895 - Installation / Warranty</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>AddressStreet1</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>Notification template</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr"/>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>895_DISPATCH_TO_USER</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>895 - Installation / Warranty</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>AddressStreet2</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>Notification template</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="inlineStr"/>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>895_DISPATCH_TO_USER</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>895 - Installation / Warranty</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>AddressZipcode</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>Notification template</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr"/>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>895_DISPATCH_TO_USER</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>895 - Installation / Warranty</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>AppointmentWindow</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>Notification template</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr"/>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>895_DISPATCH_TO_USER</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>895 - Installation / Warranty</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>AssignedUser</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
-        <is>
-          <t>Notification template</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="inlineStr"/>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>895_DISPATCH_TO_USER</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>895 - Installation / Warranty</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>AssignedUserEmail</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Notification template</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr"/>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>895_DISPATCH_TO_USER</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>895 - Installation / Warranty</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>EmailAddress</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>Notification template</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr"/>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>895_DISPATCH_TO_USER</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>895 - Installation / Warranty</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>FirstName</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>Notification template</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="inlineStr"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>895_DISPATCH_TO_USER</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>895 - Installation / Warranty</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>LastName</t>
-        </is>
-      </c>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="F14" s="10" t="inlineStr">
-        <is>
-          <t>Notification template</t>
-        </is>
-      </c>
-      <c r="G14" s="10" t="inlineStr"/>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>895_DISPATCH_TO_USER</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>895 - Installation / Warranty</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>PrimaryPhoneNumber</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>Notification template</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr"/>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>895_DISPATCH_TO_USER</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr"/>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>895 - Installation / Warranty</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>ProjectNumber</t>
-        </is>
-      </c>
-      <c r="E16" s="10" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="F16" s="10" t="inlineStr">
-        <is>
-          <t>Notification template</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A3:G16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>